<commit_message>
Fill remaining municipal contact gaps in wedding spreadsheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YHxkqbHc7V22NomUggZS9F
</commit_message>
<xml_diff>
--- a/Denmark_wedding_municipalities_2026.xlsx
+++ b/Denmark_wedding_municipalities_2026.xlsx
@@ -4056,12 +4056,12 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>post@holb.dk</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>Jernbanevej 6, 4300 Holbæk</t>
+          <t>Kanalstræde 2, 4300 Holbæk</t>
         </is>
       </c>
       <c r="K39" s="14" t="inlineStr">
@@ -6069,20 +6069,24 @@
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>99 66 70 00</t>
         </is>
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>not found</t>
+          <t>post@vesthimmerland.dk</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
-          <t>not found</t>
-        </is>
-      </c>
-      <c r="K64" s="11" t="inlineStr"/>
+          <t>Vestre Boulevard 7, 9600 Aars</t>
+        </is>
+      </c>
+      <c r="K64" s="14" t="inlineStr">
+        <is>
+          <t>https://vesthimmerland.dk/kontakt</t>
+        </is>
+      </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
           <t>not found</t>
@@ -9077,77 +9081,78 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P63" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P95" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P96" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P97" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P98" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P99" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P95" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q95" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P96" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q96" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P97" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P98" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P99" r:id="rId213"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record 17 Sep replies from town halls and agencies in wedding spreadsheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YHxkqbHc7V22NomUggZS9F
</commit_message>
<xml_diff>
--- a/Denmark_wedding_municipalities_2026.xlsx
+++ b/Denmark_wedding_municipalities_2026.xlsx
@@ -1001,7 +1001,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr"/>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>NO (17 Sep): no free slots before the end of the year</t>
+        </is>
+      </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
           <t>borgerogydelsescenter@albertslund.dk / +45 43 68 68 68</t>
@@ -1083,7 +1087,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr"/>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Auto-reply 17 Sep: received</t>
+        </is>
+      </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
           <t>vielse@brondby.dk</t>
@@ -1247,7 +1255,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr"/>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Auto-reply 17 Sep: handled within 10 working days</t>
+        </is>
+      </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
           <t>borgerservice@gribskov.dk / +45 72 49 60 00</t>
@@ -1329,7 +1341,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>NO (17 Sep): fully booked until December 2026</t>
+        </is>
+      </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
           <t>borgerservice@helsingor.dk</t>
@@ -1493,7 +1509,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Auto-reply 17 Sep: forwarded to the right department</t>
+        </is>
+      </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
           <t>skanderborg.kommune@skanderborg.dk / wedding booking +45 87 94 74 67</t>
@@ -1575,7 +1595,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>NO (17 Sep): no available dates until February 2027</t>
+        </is>
+      </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
           <t>borgerservice@lolland.dk / +45 54 67 67 67</t>
@@ -1653,7 +1677,11 @@
           <t>Emailed (sent)</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>NO (17 Sep): fully booked September, October and early November</t>
+        </is>
+      </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
           <t>vardekommune@varde.dk / +45 79 94 68 00</t>
@@ -7753,7 +7781,7 @@
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>Auto-reply: answer within 3-5 working days</t>
+          <t>Auto-reply 17 Sep: answer within 3-5 working days</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
@@ -8561,7 +8589,7 @@
       </c>
       <c r="F95" s="11" t="inlineStr">
         <is>
-          <t>Auto-reply: fully booked 2+ months, reply in 1-2 weeks</t>
+          <t>Auto-reply 17 Sep: fully booked 2+ months, reply in 1-2 weeks</t>
         </is>
       </c>
       <c r="G95" s="11" t="inlineStr">
@@ -8647,7 +8675,7 @@
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>Auto-reply: no slots until January 2027</t>
+          <t>NO (auto-reply 17 Sep): no slots until January 2027</t>
         </is>
       </c>
       <c r="G96" s="11" t="inlineStr">
@@ -9246,7 +9274,7 @@
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>Quote request sent</t>
+          <t>REPLIED 17 Sep: offers Wed 7 Oct, private registrar at a seaside hotel approx 1h south of Copenhagen Airport, EUR 1,395 all-in (Familieretshuset fee, venue, registrar, witnesses, certificates). Hold requested.</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9307,7 @@
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>Quote request sent</t>
+          <t>REPLIED 17 Sep: no town hall availability in the window; earliest end Nov / early Dec</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9344,7 @@
       </c>
       <c r="G4" s="20" t="inlineStr">
         <is>
-          <t>Quote request sent</t>
+          <t>Auto-reply 17 Sep: will respond within 24 hours</t>
         </is>
       </c>
     </row>
@@ -9349,7 +9377,7 @@
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>Quote request sent</t>
+          <t>REPLIED 17 Sep: no dates 28 Sep-7 Oct; earliest mid/late Nov; full service EUR 850</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix agency reply statuses in wedding spreadsheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YHxkqbHc7V22NomUggZS9F
</commit_message>
<xml_diff>
--- a/Denmark_wedding_municipalities_2026.xlsx
+++ b/Denmark_wedding_municipalities_2026.xlsx
@@ -9274,7 +9274,7 @@
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>REPLIED 17 Sep: offers Wed 7 Oct, private registrar at a seaside hotel approx 1h south of Copenhagen Airport, EUR 1,395 all-in (Familieretshuset fee, venue, registrar, witnesses, certificates). Hold requested.</t>
+          <t>Auto-reply 17 Sep: will respond within 24 hours</t>
         </is>
       </c>
     </row>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="G4" s="20" t="inlineStr">
         <is>
-          <t>Auto-reply 17 Sep: will respond within 24 hours</t>
+          <t>REPLIED 17 Sep: offers Wed 7 Oct, private registrar at a seaside hotel approx 1h south of Copenhagen Airport, EUR 1,395 all-in (Familieretshuset fee, venue, registrar, witnesses, certificates). Hold requested.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark Frederikssund as contacted in wedding spreadsheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YHxkqbHc7V22NomUggZS9F
</commit_message>
<xml_diff>
--- a/Denmark_wedding_municipalities_2026.xlsx
+++ b/Denmark_wedding_municipalities_2026.xlsx
@@ -2000,9 +2000,9 @@
           <t>Frederikssund, 40 km NW of Copenhagen</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>Not contacted</t>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Emailed (sent)</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr"/>

</xml_diff>